<commit_message>
Fix Artikelnummer 612/16 and remove (Kopie) from short names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDtqvNwYT39iZFKv5Z4iEs
</commit_message>
<xml_diff>
--- a/Artikel_Gourmet_ohne_Varianten.xlsx
+++ b/Artikel_Gourmet_ohne_Varianten.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ15"/>
+  <dimension ref="A1:AJ16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -638,7 +638,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>4200000000000063</t>
+          <t>9284870000000166</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -648,18 +648,18 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Hähnchen Erdnuss</t>
+          <t>Salat Garn.-Mango</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Hähnchen Erdnuss</t>
+          <t>Salat Garn.-Mango</t>
         </is>
       </c>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>602.</t>
+          <t>16.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -684,7 +684,7 @@
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>602,</t>
+          <t>16,</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -759,11 +759,11 @@
         </is>
       </c>
       <c r="AI2" s="4" t="n">
-        <v>210</v>
+        <v>10</v>
       </c>
       <c r="AJ2" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:06:24</t>
+          <t>2026-09-30 10:02:15</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4200000000000062</t>
+          <t>4200000000000063</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -785,18 +785,18 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Hähnchen Soja</t>
+          <t>Gourmet - Hähnchen Erdnuss</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Hähnchen Soja</t>
+          <t>Hähnchen Erdnuss</t>
         </is>
       </c>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>601.</t>
+          <t>602.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -821,7 +821,7 @@
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>601,</t>
+          <t>602,</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="AJ3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:06:23</t>
+          <t>2026-10-07 10:06:24</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>9284870000000186</t>
+          <t>4200000000000062</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -922,18 +922,18 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Hähnchen</t>
+          <t>Gourmet - Hähnchen Soja</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Hähnchen Curry</t>
+          <t>Hähnchen Soja</t>
         </is>
       </c>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>603.</t>
+          <t>601.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -958,7 +958,7 @@
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>603,</t>
+          <t>601,</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="AJ4" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:06:24</t>
+          <t>2026-10-07 10:06:23</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4200000000000065</t>
+          <t>9284870000000186</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1059,18 +1059,18 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Pan. Hähnchen (Kopie) (Kopie)</t>
+          <t>Gourmet - Hähnchen</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Paniert Erdnuss</t>
+          <t>Hähnchen Curry</t>
         </is>
       </c>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>613.</t>
+          <t>603.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1095,7 +1095,7 @@
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>612,</t>
+          <t>603,</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>14.5</v>
+        <v>13.9</v>
       </c>
       <c r="T5" s="2" t="n"/>
       <c r="U5" s="2" t="n"/>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="AI5" s="4" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="AJ5" s="6" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>4200000000000064</t>
+          <t>4200000000000065</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1196,18 +1196,18 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Pan. Hähnchen (Kopie)</t>
+          <t>Gourmet - Pan. Hähnchen</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Paniert Curry</t>
+          <t>Paniert Erdnuss</t>
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>613.</t>
+          <t>612.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>613,</t>
+          <t>612,</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>9284870000000187</t>
+          <t>4200000000000064</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1338,13 +1338,13 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Paniert Soja</t>
+          <t>Paniert Curry</t>
         </is>
       </c>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>611.</t>
+          <t>613.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -1369,7 +1369,7 @@
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>611,</t>
+          <t>613,</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>9284870000000188</t>
+          <t>9284870000000187</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1470,18 +1470,18 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Teriy. Chicken</t>
+          <t>Gourmet - Pan. Hähnchen</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Teriy. Chicken Soja</t>
+          <t>Paniert Soja</t>
         </is>
       </c>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>621.</t>
+          <t>611.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1506,7 +1506,7 @@
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>621,</t>
+          <t>611,</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1521,7 +1521,7 @@
         <v>0</v>
       </c>
       <c r="S8" s="5" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="n"/>
@@ -1581,11 +1581,11 @@
         </is>
       </c>
       <c r="AI8" s="4" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="AJ8" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:27:53</t>
+          <t>2026-10-07 10:06:24</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>9284870000000189</t>
+          <t>9284870000000188</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1607,18 +1607,18 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Kn. Ente Soja</t>
+          <t>Gourmet - Teriy. Chicken</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Kn. Ente Soja</t>
+          <t>Teriy. Chicken Soja</t>
         </is>
       </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>631.</t>
+          <t>621.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1643,7 +1643,7 @@
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>631,</t>
+          <t>621,</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1658,7 +1658,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="5" t="n">
-        <v>15.5</v>
+        <v>14.9</v>
       </c>
       <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="n"/>
@@ -1718,11 +1718,11 @@
         </is>
       </c>
       <c r="AI9" s="4" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="AJ9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:06:25</t>
+          <t>2026-10-07 10:27:53</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>4200000000000067</t>
+          <t>9284870000000189</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1744,18 +1744,18 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Kn. Ente Erdnuss</t>
+          <t>Gourmet - Kn. Ente Soja</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Kn. Ente Erdnuss</t>
+          <t>Kn. Ente Soja</t>
         </is>
       </c>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>632.</t>
+          <t>631.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>632,</t>
+          <t>631,</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>4200000000000066</t>
+          <t>4200000000000067</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1881,18 +1881,18 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Kn. Ente Curry</t>
+          <t>Gourmet - Kn. Ente Erdnuss</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Kn. Ente Curry</t>
+          <t>Kn. Ente Erdnuss</t>
         </is>
       </c>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>633.</t>
+          <t>632.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1917,7 +1917,7 @@
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>633,</t>
+          <t>632,</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>9284870000000190</t>
+          <t>4200000000000066</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2018,18 +2018,18 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Rind</t>
+          <t>Gourmet - Kn. Ente Curry</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Rind Soja</t>
+          <t>Kn. Ente Curry</t>
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>641.</t>
+          <t>633.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -2054,7 +2054,7 @@
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>641,</t>
+          <t>633,</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -2069,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="S12" s="5" t="n">
-        <v>14.9</v>
+        <v>15.5</v>
       </c>
       <c r="T12" s="2" t="n"/>
       <c r="U12" s="2" t="n"/>
@@ -2129,11 +2129,11 @@
         </is>
       </c>
       <c r="AI12" s="4" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="AJ12" s="6" t="inlineStr">
         <is>
-          <t>2026-10-07 10:27:53</t>
+          <t>2026-10-07 10:06:25</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>9284870000000191</t>
+          <t>9284870000000190</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2155,18 +2155,18 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Garn.</t>
+          <t>Gourmet - Rind</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Garnele Soja</t>
+          <t>Rind Soja</t>
         </is>
       </c>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>651.</t>
+          <t>641.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -2191,7 +2191,7 @@
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>651,</t>
+          <t>641,</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2206,7 +2206,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="5" t="n">
-        <v>15.9</v>
+        <v>14.9</v>
       </c>
       <c r="T13" s="2" t="n"/>
       <c r="U13" s="2" t="n"/>
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="AI13" s="4" t="n">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="AJ13" s="6" t="inlineStr">
         <is>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>9284870000000192</t>
+          <t>9284870000000191</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2292,18 +2292,18 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Lachs</t>
+          <t>Gourmet - Garn.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Lachs Soja</t>
+          <t>Garnele Soja</t>
         </is>
       </c>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>661.</t>
+          <t>651.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -2328,7 +2328,7 @@
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>661,</t>
+          <t>651,</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -2343,7 +2343,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="5" t="n">
-        <v>16.9</v>
+        <v>15.9</v>
       </c>
       <c r="T14" s="2" t="n"/>
       <c r="U14" s="2" t="n"/>
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="AI14" s="4" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="AJ14" s="6" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>9284870000000193</t>
+          <t>9284870000000192</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2429,18 +2429,18 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Gourmet - Tofu</t>
+          <t>Gourmet - Lachs</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tofu Soja</t>
+          <t>Lachs Soja</t>
         </is>
       </c>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>671.</t>
+          <t>661.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -2465,7 +2465,7 @@
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>671,</t>
+          <t>661,</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2480,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="5" t="n">
-        <v>13.5</v>
+        <v>16.9</v>
       </c>
       <c r="T15" s="2" t="n"/>
       <c r="U15" s="2" t="n"/>
@@ -2540,15 +2540,151 @@
         </is>
       </c>
       <c r="AI15" s="4" t="n">
+        <v>270</v>
+      </c>
+      <c r="AJ15" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-07 10:27:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>maiwokzokasse@gmail.com</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>9284870000000193</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Gourmet - Tofu</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Tofu Soja</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>671.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>9284870000000047</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>671,</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Stk</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="5" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
+      <c r="V16" s="2" t="n"/>
+      <c r="W16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="3" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="AA16" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB16" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC16" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AD16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="AI16" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="AJ15" s="6" t="inlineStr">
+      <c r="AJ16" s="6" t="inlineStr">
         <is>
           <t>2026-10-07 10:27:53</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17"/>
     <row r="18"/>
     <row r="19"/>

</xml_diff>